<commit_message>
fixes field order on data and metadata
</commit_message>
<xml_diff>
--- a/data-raw/metadata/clear_redd_reach_river_mile_reference_metadata.xlsx
+++ b/data-raw/metadata/clear_redd_reach_river_mile_reference_metadata.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Badhia\Documents\git\jpe-clear-adult-edi\data-raw\metadata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9294E409-60AE-45B2-BCCD-736AE3BC521C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{212A4391-06FB-4193-A53E-B728E7F359C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4360" yWindow="1180" windowWidth="19200" windowHeight="11170" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -109,9 +109,6 @@
     <t>reach_number</t>
   </si>
   <si>
-    <t>years</t>
-  </si>
-  <si>
     <t>River mile where reach starts</t>
   </si>
   <si>
@@ -119,9 +116,6 @@
   </si>
   <si>
     <t>Survey reach number</t>
-  </si>
-  <si>
-    <t>Years when river mile extent applies to</t>
   </si>
   <si>
     <t>rivermile</t>
@@ -146,6 +140,12 @@
   </si>
   <si>
     <t>1</t>
+  </si>
+  <si>
+    <t>year_extent</t>
+  </si>
+  <si>
+    <t>Year range when river mile extent applies to</t>
   </si>
 </sst>
 </file>
@@ -226,7 +226,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -254,7 +254,6 @@
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="49" fontId="6" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -544,39 +543,29 @@
       <c r="Z1" s="7"/>
     </row>
     <row r="2" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="13" t="s">
-        <v>24</v>
+      <c r="A2" s="4" t="s">
+        <v>38</v>
       </c>
-      <c r="B2" s="13" t="s">
-        <v>28</v>
+      <c r="B2" s="4" t="s">
+        <v>39</v>
       </c>
-      <c r="C2" s="13" t="s">
-        <v>13</v>
+      <c r="C2" s="4" t="s">
+        <v>19</v>
       </c>
       <c r="D2" s="14" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
-      <c r="E2" s="13" t="s">
-        <v>14</v>
+      <c r="E2" s="4" t="s">
+        <v>20</v>
       </c>
-      <c r="F2" s="15" t="s">
-        <v>13</v>
-      </c>
-      <c r="G2" s="15" t="s">
-        <v>32</v>
-      </c>
-      <c r="H2" s="15" t="s">
-        <v>33</v>
-      </c>
-      <c r="I2" s="14"/>
-      <c r="J2" s="15"/>
-      <c r="K2" s="14"/>
-      <c r="L2" s="16" t="s">
-        <v>35</v>
-      </c>
-      <c r="M2" s="16" t="s">
-        <v>36</v>
-      </c>
+      <c r="F2" s="6"/>
+      <c r="G2" s="6"/>
+      <c r="H2" s="6"/>
+      <c r="I2" s="5"/>
+      <c r="J2" s="6"/>
+      <c r="K2" s="5"/>
+      <c r="L2" s="6"/>
+      <c r="M2" s="6"/>
       <c r="N2" s="7"/>
       <c r="O2" s="7"/>
       <c r="P2" s="7"/>
@@ -593,9 +582,9 @@
     </row>
     <row r="3" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A3" s="13" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
-      <c r="B3" s="13" t="s">
+      <c r="B3" s="4" t="s">
         <v>29</v>
       </c>
       <c r="C3" s="13" t="s">
@@ -614,7 +603,7 @@
         <v>32</v>
       </c>
       <c r="H3" s="15" t="s">
-        <v>33</v>
+        <v>18</v>
       </c>
       <c r="I3" s="14"/>
       <c r="J3" s="15"/>
@@ -623,7 +612,7 @@
         <v>37</v>
       </c>
       <c r="M3" s="16" t="s">
-        <v>38</v>
+        <v>21</v>
       </c>
       <c r="N3" s="7"/>
       <c r="O3" s="7"/>
@@ -641,16 +630,16 @@
     </row>
     <row r="4" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A4" s="13" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
-      <c r="B4" s="4" t="s">
-        <v>30</v>
+      <c r="B4" s="13" t="s">
+        <v>27</v>
       </c>
       <c r="C4" s="13" t="s">
         <v>13</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E4" s="13" t="s">
         <v>14</v>
@@ -659,19 +648,19 @@
         <v>13</v>
       </c>
       <c r="G4" s="15" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="H4" s="15" t="s">
-        <v>18</v>
+        <v>31</v>
       </c>
       <c r="I4" s="14"/>
       <c r="J4" s="15"/>
       <c r="K4" s="14"/>
       <c r="L4" s="16" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="M4" s="16" t="s">
-        <v>21</v>
+        <v>34</v>
       </c>
       <c r="N4" s="7"/>
       <c r="O4" s="7"/>
@@ -688,29 +677,39 @@
       <c r="Z4" s="7"/>
     </row>
     <row r="5" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A5" s="4" t="s">
-        <v>27</v>
+      <c r="A5" s="13" t="s">
+        <v>25</v>
       </c>
-      <c r="B5" s="4" t="s">
-        <v>31</v>
+      <c r="B5" s="13" t="s">
+        <v>28</v>
       </c>
-      <c r="C5" s="4" t="s">
-        <v>19</v>
+      <c r="C5" s="13" t="s">
+        <v>13</v>
       </c>
       <c r="D5" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="E5" s="4" t="s">
-        <v>20</v>
+      <c r="E5" s="13" t="s">
+        <v>14</v>
       </c>
-      <c r="F5" s="6"/>
-      <c r="G5" s="6"/>
-      <c r="H5" s="6"/>
-      <c r="I5" s="5"/>
-      <c r="J5" s="6"/>
-      <c r="K5" s="5"/>
-      <c r="L5" s="17"/>
-      <c r="M5" s="6"/>
+      <c r="F5" s="15" t="s">
+        <v>13</v>
+      </c>
+      <c r="G5" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="H5" s="15" t="s">
+        <v>31</v>
+      </c>
+      <c r="I5" s="14"/>
+      <c r="J5" s="15"/>
+      <c r="K5" s="14"/>
+      <c r="L5" s="16" t="s">
+        <v>35</v>
+      </c>
+      <c r="M5" s="16" t="s">
+        <v>36</v>
+      </c>
       <c r="N5" s="7"/>
       <c r="O5" s="7"/>
       <c r="P5" s="7"/>
@@ -724,34 +723,6 @@
       <c r="X5" s="7"/>
       <c r="Y5" s="7"/>
       <c r="Z5" s="7"/>
-    </row>
-    <row r="6" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A6" s="4"/>
-      <c r="B6" s="4"/>
-      <c r="C6" s="4"/>
-      <c r="D6" s="5"/>
-      <c r="E6" s="4"/>
-      <c r="F6" s="6"/>
-      <c r="G6" s="6"/>
-      <c r="H6" s="6"/>
-      <c r="I6" s="5"/>
-      <c r="J6" s="6"/>
-      <c r="K6" s="5"/>
-      <c r="L6" s="10"/>
-      <c r="M6" s="6"/>
-      <c r="N6" s="7"/>
-      <c r="O6" s="7"/>
-      <c r="P6" s="7"/>
-      <c r="Q6" s="7"/>
-      <c r="R6" s="7"/>
-      <c r="S6" s="7"/>
-      <c r="T6" s="7"/>
-      <c r="U6" s="7"/>
-      <c r="V6" s="7"/>
-      <c r="W6" s="7"/>
-      <c r="X6" s="7"/>
-      <c r="Y6" s="7"/>
-      <c r="Z6" s="7"/>
     </row>
     <row r="7" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A7" s="4"/>
@@ -28321,16 +28292,16 @@
     </row>
   </sheetData>
   <dataValidations count="4">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C48:C991 C24:C36 C1:C22" xr:uid="{00000000-0002-0000-0000-000002000000}">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C48:C991 C24:C36 C1:C5 C7:C22" xr:uid="{00000000-0002-0000-0000-000002000000}">
       <formula1>"nominal,ordinal,interval,ratio,dateTime"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="E24:E991 E1:E22" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="E24:E991 E1:E5 E7:E22" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"text,enumerated,dateTime,numeric"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="F24:F991 F1:F22" xr:uid="{00000000-0002-0000-0000-000001000000}">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="F24:F991 F1:F5 F7:F22" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>"ratio,interval"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="H24:H991 H1:H22" xr:uid="{00000000-0002-0000-0000-000003000000}">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="H24:H991 H1:H5 H7:H22" xr:uid="{00000000-0002-0000-0000-000003000000}">
       <formula1>"natural,whole,integer,real"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
updates rier mile referencec metadata
</commit_message>
<xml_diff>
--- a/data-raw/metadata/clear_redd_reach_river_mile_reference_metadata.xlsx
+++ b/data-raw/metadata/clear_redd_reach_river_mile_reference_metadata.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Badhia\Documents\git\jpe-clear-adult-edi\data-raw\metadata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{212A4391-06FB-4193-A53E-B728E7F359C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2DB52B2-6199-4A8A-92C1-7009B5408D91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4360" yWindow="1180" windowWidth="19200" windowHeight="11170" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2990" yWindow="910" windowWidth="15280" windowHeight="11780" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="attribute" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="38">
   <si>
     <t xml:space="preserve">attribute_name </t>
   </si>
@@ -82,9 +82,6 @@
     <t>attribute_name</t>
   </si>
   <si>
-    <t>whole</t>
-  </si>
-  <si>
     <t>ordinal</t>
   </si>
   <si>
@@ -115,16 +112,10 @@
     <t>River mile where reach ends</t>
   </si>
   <si>
-    <t>Survey reach number</t>
-  </si>
-  <si>
     <t>rivermile</t>
   </si>
   <si>
     <t>integer</t>
-  </si>
-  <si>
-    <t>reach</t>
   </si>
   <si>
     <t>1.77</t>
@@ -146,6 +137,9 @@
   </si>
   <si>
     <t>Year range when river mile extent applies to</t>
+  </si>
+  <si>
+    <t>Survey reach number. Levels = c("1", "2", "3", "4", "5A", "5B", "6", "UCC RST", "5C", "6A", "6B", "7", "5")</t>
   </si>
 </sst>
 </file>
@@ -544,19 +538,19 @@
     </row>
     <row r="2" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A2" s="4" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D2" s="14" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F2" s="6"/>
       <c r="G2" s="6"/>
@@ -582,37 +576,31 @@
     </row>
     <row r="3" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A3" s="13" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="C3" s="13" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="D3" s="14" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E3" s="13" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
-      <c r="F3" s="15" t="s">
-        <v>13</v>
-      </c>
-      <c r="G3" s="15" t="s">
-        <v>32</v>
-      </c>
-      <c r="H3" s="15" t="s">
-        <v>18</v>
-      </c>
+      <c r="F3" s="15"/>
+      <c r="G3" s="15"/>
+      <c r="H3" s="15"/>
       <c r="I3" s="14"/>
       <c r="J3" s="15"/>
       <c r="K3" s="14"/>
       <c r="L3" s="16" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="M3" s="16" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="N3" s="7"/>
       <c r="O3" s="7"/>
@@ -630,16 +618,16 @@
     </row>
     <row r="4" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A4" s="13" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B4" s="13" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C4" s="13" t="s">
         <v>13</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E4" s="13" t="s">
         <v>14</v>
@@ -648,19 +636,19 @@
         <v>13</v>
       </c>
       <c r="G4" s="15" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="H4" s="15" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="I4" s="14"/>
       <c r="J4" s="15"/>
       <c r="K4" s="14"/>
       <c r="L4" s="16" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="M4" s="16" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="N4" s="7"/>
       <c r="O4" s="7"/>
@@ -678,16 +666,16 @@
     </row>
     <row r="5" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A5" s="13" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B5" s="13" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C5" s="13" t="s">
         <v>13</v>
       </c>
       <c r="D5" s="14" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E5" s="13" t="s">
         <v>14</v>
@@ -696,19 +684,19 @@
         <v>13</v>
       </c>
       <c r="G5" s="15" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="H5" s="15" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="I5" s="14"/>
       <c r="J5" s="15"/>
       <c r="K5" s="14"/>
       <c r="L5" s="16" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="M5" s="16" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="N5" s="7"/>
       <c r="O5" s="7"/>

</xml_diff>